<commit_message>
FINALMENTE CONSEGUI CONSERTAR A BCT DO CROSS-SELLING!
</commit_message>
<xml_diff>
--- a/dados_entrada/Analise_Comercial_Completa.xlsx
+++ b/dados_entrada/Analise_Comercial_Completa.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m.rafael\Desktop\PROJETO_COMISSOES_V2\dados_entrada\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meu Computador\Desktop\Clean Trabalho\PROJETO_COMISSOES_V2\dados_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0689D9C8-A675-4D7A-9641-E77202A2D472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CA0BE457-E36A-4D33-9EB8-EC119843CD00}"/>
+    <workbookView xWindow="22935" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="56">
   <si>
     <t>100002</t>
   </si>
@@ -172,12 +171,42 @@
   </si>
   <si>
     <t>XCD</t>
+  </si>
+  <si>
+    <t>400001</t>
+  </si>
+  <si>
+    <t>448001</t>
+  </si>
+  <si>
+    <t>2025-08-10</t>
+  </si>
+  <si>
+    <t>SAMANTA</t>
+  </si>
+  <si>
+    <t>Hidrologia</t>
+  </si>
+  <si>
+    <t>Medidor de Vazão Fixo</t>
+  </si>
+  <si>
+    <t>ADP</t>
+  </si>
+  <si>
+    <t>PROD400001</t>
+  </si>
+  <si>
+    <t>Produto de Teste - Processo 400001</t>
+  </si>
+  <si>
+    <t>MATEUS BORRO MACHADO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -230,11 +259,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,8 +578,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D438093-7464-46A3-87DA-40F4B4EBC2C2}">
-  <dimension ref="A1:X3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:X4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
@@ -560,9 +590,9 @@
     <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.5703125" bestFit="1" customWidth="1"/>
@@ -666,10 +696,10 @@
         <v>4</v>
       </c>
       <c r="F2">
-        <v>12000</v>
+        <v>50</v>
       </c>
       <c r="G2">
-        <v>13200</v>
+        <v>50</v>
       </c>
       <c r="H2" t="s">
         <v>5</v>
@@ -730,14 +760,14 @@
       <c r="D3" t="s">
         <v>3</v>
       </c>
-      <c r="E3" t="s">
-        <v>4</v>
+      <c r="E3" s="2">
+        <v>45885</v>
       </c>
       <c r="F3">
-        <v>12000</v>
+        <v>20</v>
       </c>
       <c r="G3">
-        <v>13200</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
         <v>5</v>
@@ -782,10 +812,82 @@
         <v>18</v>
       </c>
       <c r="W3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="2">
+        <v>45870</v>
+      </c>
+      <c r="F4">
+        <v>70</v>
+      </c>
+      <c r="G4">
+        <v>70</v>
+      </c>
+      <c r="H4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" t="s">
+        <v>52</v>
+      </c>
+      <c r="N4" t="s">
+        <v>10</v>
+      </c>
+      <c r="O4" t="s">
+        <v>11</v>
+      </c>
+      <c r="P4" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>13</v>
+      </c>
+      <c r="R4" t="s">
+        <v>14</v>
+      </c>
+      <c r="S4" t="s">
+        <v>15</v>
+      </c>
+      <c r="T4" t="s">
+        <v>53</v>
+      </c>
+      <c r="U4" t="s">
+        <v>54</v>
+      </c>
+      <c r="V4" t="s">
+        <v>18</v>
+      </c>
+      <c r="W4" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>